<commit_message>
Adiciona novos documentos de apresentação e planejamento do DUAXIS, incluindo uma proposta de apresentação em PDF e um roteiro atualizado para a apresentação. O documento "TUDO OQUE FOI FEITO" foi criado para detalhar ajustes e funcionalidades do projeto, visando melhorar a comunicação e a clareza das informações apresentadas. Essas adições têm como objetivo aprimorar a experiência de apresentação e facilitar a compreensão do projeto por stakeholders e novos membros da equipe.
</commit_message>
<xml_diff>
--- a/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
+++ b/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Esther\Documents\PROJETO - START TECH\duaxis-projeto-start-tech\DOCUMENTOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EBCDC0A-C78F-4100-BBE3-6AFF0741192F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9FB3AC-4B26-44A2-AE28-9EAB4109C5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{6FE2B4A4-5807-4032-A764-0DC1BFE9E1AF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{6FE2B4A4-5807-4032-A764-0DC1BFE9E1AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>INTERFACE</t>
   </si>
@@ -68,28 +68,35 @@
     <t>JUSTIFICATIVA</t>
   </si>
   <si>
-    <t>A estrutura visual do DUAXIS já existe, incluindo chat e renderizações específicas para alguns retornos. O que ainda pesa é integrar as funcionalidades que faltam, finalizar Financeiro, simulador/relatórios e fazer refinamentos de UX, erros, loading, estados vazios e responsividade.</t>
-  </si>
-  <si>
     <t>Já temos bases integradas de produtos, clientes, fornecedores, vendas, compras, estoque, movimentações de estoque, contas a pagar/receber e movimentações financeiras, com histórico suficiente para as análises. Também já validamos relações importantes, como reconstrução histórica de estoque. 5% para eventuais ajustes e validações finais.</t>
   </si>
   <si>
-    <t>O LLM já está integrado via Groq, temos Tool Calling, prompt de sistema, restrição de domínio e regras contra respostas repetitivas. A IA já consegue interpretar diferentes formas de perguntar e extrair períodos. Ainda faltam ampliar as ferramentas, principalmente Financeiro, histórico conversacional e testes mais extensos de robustez.</t>
-  </si>
-  <si>
-    <t>Aqui já temos bastante coisa: previsão de demanda com Random Forest, reposição, cobertura de estoque, risco de ruptura, pedidos atrasados e a análise de menor giro com comparação histórica/sazonal. Ainda faltam principalmente as análises financeiras, causas de variações e o segundo modelo preditivo planejado.</t>
-  </si>
-  <si>
-    <t>Isso já caracteriza um copiloto funcional. Porém, para chegar perto de 100%, ele precisa cobrir melhor as diferentes áreas da empresa, especialmente Financeiro + Logística, além de histórico conversacional, relatórios, simulador e maior integração das funcionalidades.</t>
-  </si>
-  <si>
-    <t>FastAPI está funcionando, temos /api/chat, integração com serviços, ML, IA e serviços logísticos. A arquitetura já começou a ser separada em ml_service, ia_service, logistica_service e periodo_service. O grande bloco que falta é financeiro_service.py, além de tratamento de erros, validações, organização/limpeza e preparação para produção.</t>
-  </si>
-  <si>
-    <t>Já existe uma camada lógica importante no prompt restringindo a IA ao domínio da Urban Style/DUAXIS, mas isso não equivale à segurança da aplicação. Ainda precisamos pensar em proteção da API, segredo da GROQ_API_KEY, validação de entrada, CORS de produção, tratamento de erros sem exposição de informações internas, limites de requisições e outras proteções adequadas ao MVP.</t>
-  </si>
-  <si>
-    <t>Ainda precisamos validar coisas como funcionamento do backend/IA em produção, variáveis de ambiente, comportamento após novos commits, erros de produção e integração completa conforme novas funcionalidades forem adicionadas.</t>
+    <t>A estrutura visual do DUAXIS já existe, incluindo chat, dashboard.
+Falta fazer refinamentos de UX, erros, loading, estados vazios e responsividade.</t>
+  </si>
+  <si>
+    <t>O LLM já está integrado via Groq, temos Tool Calling, prompt de sistema, regras contra respostas repetitivas. A IA já consegue interpretar diferentes formas de perguntar e extrair períodos, contexto de sessão ("E as despesas"). Ainda faltam testes mais extensos de robustez.</t>
+  </si>
+  <si>
+    <t>Aqui já temos bastante coisa: previsão de demanda com Random Forest, reposição, cobertura de estoque, risco de ruptura, pedidos atrasados e a análise de menor giro com comparação histórica/sazonal.</t>
+  </si>
+  <si>
+    <t>Isso já caracteriza um copiloto funcional.
+Cobertura financeiro + logística; glossário; simulador; relatório; follow-up na mesma aba; cards + fonte da análise.</t>
+  </si>
+  <si>
+    <t>FastAPI está funcionando, dashboard, horário, PDF; financeiro_service, dashboard_service, relatorio_service, glossario_service além de ML/IA/logística/período.</t>
+  </si>
+  <si>
+    <t>Há vercel.json e o README ensina a rodar local.
+Validar backend/IA no ar; variáveis de ambiente; comportamento após commit; CORS e erros em produção.</t>
+  </si>
+  <si>
+    <t>Já existe uma camada lógica importante no prompt restringindo a IA ao domínio da Urban Style/DUAXIS, mas isso não equivale à segurança da aplicação. Ainda precisamos pensar em proteção da API, segredo da GROQ_API_KEY, tratamento de erros sem exposição de informações internas, limites de requisições e outras proteções adequadas ao MVP.</t>
+  </si>
+  <si>
+    <t>VER COM A IA OQUE PODEMOS FAZER DE SEGURANÇA (USAR 3 IAS - COLOCAR CLOUD ENTRE ELAS)
+ARGUMENTOS DO QUE FOI USADO DE SEGURANÇA, BIBLIOTECA PYTHON (?)</t>
   </si>
 </sst>
 </file>
@@ -508,109 +515,141 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD167CA4-7F77-44F6-B9CA-FED0DC092A4E}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.109375" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" customWidth="1"/>
+    <col min="4" max="4" width="46.140625" customWidth="1"/>
+    <col min="5" max="5" width="57.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="5">
         <v>46265</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5">
+        <v>46274</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3">
         <v>0.7</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C2" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3">
         <v>0.95</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C3" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3">
         <v>0.7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3">
+        <v>0.85</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="3">
         <v>0.65</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3">
+        <v>0.86</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="3">
         <v>0.6</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3">
+        <v>0.86</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>0.65</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="3">
         <v>0.5</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="C8" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="3">
         <v>0.15</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>15</v>
+      <c r="C9" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementa sistema de autenticação para o gestor, adicionando endpoints de login e verificação de sessão no backend. Inclui lógica de segurança com HMAC para garantir a integridade dos dados e atualiza o frontend para gerenciar a tela de login do gestor. Além disso, ajusta o CSS para estilizar a interface de login. Essa atualização visa melhorar a segurança e a experiência do usuário ao acessar o sistema DUAXIS.
</commit_message>
<xml_diff>
--- a/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
+++ b/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Esther\Documents\PROJETO - START TECH\duaxis-projeto-start-tech\DOCUMENTOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9FB3AC-4B26-44A2-AE28-9EAB4109C5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3EC663-33D4-44B2-8608-ADABB47173CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{6FE2B4A4-5807-4032-A764-0DC1BFE9E1AF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>INTERFACE</t>
   </si>
@@ -92,11 +92,60 @@
 Validar backend/IA no ar; variáveis de ambiente; comportamento após commit; CORS e erros em produção.</t>
   </si>
   <si>
-    <t>Já existe uma camada lógica importante no prompt restringindo a IA ao domínio da Urban Style/DUAXIS, mas isso não equivale à segurança da aplicação. Ainda precisamos pensar em proteção da API, segredo da GROQ_API_KEY, tratamento de erros sem exposição de informações internas, limites de requisições e outras proteções adequadas ao MVP.</t>
-  </si>
-  <si>
-    <t>VER COM A IA OQUE PODEMOS FAZER DE SEGURANÇA (USAR 3 IAS - COLOCAR CLOUD ENTRE ELAS)
-ARGUMENTOS DO QUE FOI USADO DE SEGURANÇA, BIBLIOTECA PYTHON (?)</t>
+    <t>Tratamos segurança em camadas. A chave da Groq não fica no frontend, usa dotenv. Para o sistema como produto, o passlib entra na tela de login: a senha do gestor nunca é armazenada em claro, e o chat só responde com sessão válida. O cryptography entra nas bases: HMAC nos CSVs para detectar manipulação dos dados da Urban Style. Fraude contábil em si não é papel do copiloto — o DUAXIS não substitui o ERP. O que ele garante é: quem pergunta está autenticado, a fonte não foi adulterada, e o número não é gerado pela IA</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>passlib - Ideia: a senha nunca viaja nem fica</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> gravada como 123456. O que o sistema guarda é um hash (texto irreversível). No login, o passlib hasheia o que a pessoa digitou e compara com o hash salvo. Pedir para o usuário trocar a cada X meses a senha
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">cryptography — integridade das bases
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Ideia: os indicadores saem de backend/dados/*.csv. Se alguém abrir vendas_urban_style.csv e alterar um valor_liquido, o copiloto mentiria com cara de verdade. HMAC detecta isso.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Fazer tela de Login e Senha, ver se tem algo</t>
+  </si>
+  <si>
+    <t>Fazer um video de fazer login em senha para mostrar na apresentação</t>
   </si>
 </sst>
 </file>
@@ -161,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -180,6 +229,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,17 +567,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD167CA4-7F77-44F6-B9CA-FED0DC092A4E}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" customWidth="1"/>
-    <col min="4" max="4" width="46.140625" customWidth="1"/>
-    <col min="5" max="5" width="57.5703125" customWidth="1"/>
+    <col min="3" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="46.140625" customWidth="1"/>
+    <col min="7" max="7" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="5">
         <v>46265</v>
@@ -533,11 +585,17 @@
       <c r="C1" s="5">
         <v>46274</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5">
+        <v>46286</v>
+      </c>
+      <c r="E1" s="5">
+        <v>46300</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -547,11 +605,17 @@
       <c r="C2" s="3">
         <v>0.88</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -561,11 +625,17 @@
       <c r="C3" s="3">
         <v>0.95</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -575,11 +645,17 @@
       <c r="C4" s="3">
         <v>0.85</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3">
+        <v>0.9</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.9</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -589,11 +665,17 @@
       <c r="C5" s="3">
         <v>0.86</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -603,11 +685,17 @@
       <c r="C6" s="3">
         <v>0.86</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -617,11 +705,17 @@
       <c r="C7" s="3">
         <v>0.88</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -631,11 +725,17 @@
       <c r="C8" s="3">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="210" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
@@ -645,11 +745,27 @@
       <c r="C9" s="3">
         <v>0.15</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>17</v>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza o roteiro de apresentação do DUAXIS, substituindo "gestor" por "usuário" para refletir melhor a interação com o sistema. Adiciona novos vídeos de login e permissões, além de implementar uma página inicial que redireciona para a tela de login. Melhora a estrutura do frontend com novas seções e ajustes de CSS para a interface de login e perfil do usuário, visando aprimorar a experiência do usuário ao acessar e interagir com o sistema.
</commit_message>
<xml_diff>
--- a/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
+++ b/DOCUMENTOS/PORCENTAGEM DAS ENTREGAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Esther\Documents\PROJETO - START TECH\duaxis-projeto-start-tech\DOCUMENTOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3EC663-33D4-44B2-8608-ADABB47173CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F833BB58-BE08-4488-ADAE-630997DAF3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{6FE2B4A4-5807-4032-A764-0DC1BFE9E1AF}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{6FE2B4A4-5807-4032-A764-0DC1BFE9E1AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>INTERFACE</t>
   </si>
@@ -140,12 +140,6 @@
       <t xml:space="preserve">Ideia: os indicadores saem de backend/dados/*.csv. Se alguém abrir vendas_urban_style.csv e alterar um valor_liquido, o copiloto mentiria com cara de verdade. HMAC detecta isso.
 </t>
     </r>
-  </si>
-  <si>
-    <t>Fazer tela de Login e Senha, ver se tem algo</t>
-  </si>
-  <si>
-    <t>Fazer um video de fazer login em senha para mostrar na apresentação</t>
   </si>
 </sst>
 </file>
@@ -567,17 +561,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD167CA4-7F77-44F6-B9CA-FED0DC092A4E}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="10.28515625" customWidth="1"/>
-    <col min="6" max="6" width="46.140625" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="10.33203125" customWidth="1"/>
+    <col min="6" max="6" width="46.109375" customWidth="1"/>
     <col min="7" max="7" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="5">
         <v>46265</v>
@@ -595,7 +589,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -615,7 +609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -635,7 +629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -655,7 +649,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -675,7 +669,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -695,7 +689,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -715,7 +709,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -735,7 +729,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="210" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
@@ -756,16 +750,6 @@
       </c>
       <c r="G9" s="7" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G11" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>